<commit_message>
2nd updated assiggnmennt showing and storing file size and file then transffer files
</commit_message>
<xml_diff>
--- a/excel_folder/customers.xlsx
+++ b/excel_folder/customers.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ony43\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C43ACBD-2DDE-455C-8244-895084F1CA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="95">
   <si>
     <t>customer_id</t>
   </si>
@@ -179,13 +185,133 @@
   </si>
   <si>
     <t>Address line 9, City 9</t>
+  </si>
+  <si>
+    <t>CUST1010</t>
+  </si>
+  <si>
+    <t>CUST1011</t>
+  </si>
+  <si>
+    <t>CUST1012</t>
+  </si>
+  <si>
+    <t>CUST1013</t>
+  </si>
+  <si>
+    <t>CUST1014</t>
+  </si>
+  <si>
+    <t>Customer_10</t>
+  </si>
+  <si>
+    <t>Customer_11</t>
+  </si>
+  <si>
+    <t>Customer_12</t>
+  </si>
+  <si>
+    <t>Customer_13</t>
+  </si>
+  <si>
+    <t>Customer_14</t>
+  </si>
+  <si>
+    <t>Customer_15</t>
+  </si>
+  <si>
+    <t>Customer_16</t>
+  </si>
+  <si>
+    <t>Customer_17</t>
+  </si>
+  <si>
+    <t>Customer_18</t>
+  </si>
+  <si>
+    <t>Customer_19</t>
+  </si>
+  <si>
+    <t>CUST1015</t>
+  </si>
+  <si>
+    <t>CUST1016</t>
+  </si>
+  <si>
+    <t>CUST1017</t>
+  </si>
+  <si>
+    <t>CUST1018</t>
+  </si>
+  <si>
+    <t>CUST1019</t>
+  </si>
+  <si>
+    <t>0170000010</t>
+  </si>
+  <si>
+    <t>Address line 9, City 10</t>
+  </si>
+  <si>
+    <t>0170000011</t>
+  </si>
+  <si>
+    <t>Address line 9, City 11</t>
+  </si>
+  <si>
+    <t>0170000012</t>
+  </si>
+  <si>
+    <t>Address line 9, City 12</t>
+  </si>
+  <si>
+    <t>0170000013</t>
+  </si>
+  <si>
+    <t>Address line 9, City 13</t>
+  </si>
+  <si>
+    <t>0170000014</t>
+  </si>
+  <si>
+    <t>Address line 9, City 14</t>
+  </si>
+  <si>
+    <t>0170000015</t>
+  </si>
+  <si>
+    <t>Address line 9, City 15</t>
+  </si>
+  <si>
+    <t>0170000016</t>
+  </si>
+  <si>
+    <t>Address line 9, City 16</t>
+  </si>
+  <si>
+    <t>0170000017</t>
+  </si>
+  <si>
+    <t>Address line 9, City 17</t>
+  </si>
+  <si>
+    <t>0170000018</t>
+  </si>
+  <si>
+    <t>Address line 9, City 18</t>
+  </si>
+  <si>
+    <t>0170000019</t>
+  </si>
+  <si>
+    <t>Address line 9, City 19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,6 +323,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -248,13 +380,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -292,7 +432,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -326,6 +466,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -360,9 +501,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -535,11 +677,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,7 +698,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -573,7 +715,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -590,7 +732,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -607,7 +749,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -624,7 +766,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -641,7 +783,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -658,7 +800,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -675,7 +817,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -692,7 +834,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -709,7 +851,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -726,7 +868,178 @@
         <v>54</v>
       </c>
     </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>